<commit_message>
Add Saanjh Choker Set (₹6,999), fix product IDs
</commit_message>
<xml_diff>
--- a/business/pricing-calculator.xlsx
+++ b/business/pricing-calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D3566A23-DEF6-419B-B116-A4BEFFE36388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9C81922F-5FCE-4D10-B68D-A8049626A2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Product Name</t>
   </si>
@@ -34,12 +34,6 @@
     <t>Price Point (rounded)</t>
   </si>
   <si>
-    <t>Kaveri Necklace Set</t>
-  </si>
-  <si>
-    <t>Raahi Necklace Set</t>
-  </si>
-  <si>
     <t>Supplier Cost</t>
   </si>
   <si>
@@ -62,6 +56,15 @@
   </si>
   <si>
     <t>Profit</t>
+  </si>
+  <si>
+    <t>Kaveri</t>
+  </si>
+  <si>
+    <t>Raahi</t>
+  </si>
+  <si>
+    <t>Saanjh</t>
   </si>
 </sst>
 </file>
@@ -930,10 +933,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692CD7B8-8219-4BAB-B946-0AD4DC2CA2E3}">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.44140625" bestFit="1" customWidth="1"/>
@@ -952,31 +955,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>2</v>
@@ -987,7 +990,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>450</v>
@@ -1032,7 +1035,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>1240</v>
@@ -1073,6 +1076,51 @@
       <c r="L3" t="str">
         <f>"₹"&amp;TEXT(G3,"#,##0")</f>
         <v>₹5,999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4">
+        <v>1495</v>
+      </c>
+      <c r="C4">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>150</v>
+      </c>
+      <c r="E4">
+        <f>B4+C4+D4</f>
+        <v>1670</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <f>ROUNDUP((E4*F4)/500,0)*500-1</f>
+        <v>6999</v>
+      </c>
+      <c r="H4">
+        <f>G4*2%</f>
+        <v>139.97999999999999</v>
+      </c>
+      <c r="I4">
+        <f>G4-H4</f>
+        <v>6859.02</v>
+      </c>
+      <c r="J4">
+        <f>I4-E4</f>
+        <v>5189.0200000000004</v>
+      </c>
+      <c r="K4" s="1">
+        <f>J4/G4</f>
+        <v>0.74139448492641813</v>
+      </c>
+      <c r="L4" t="str">
+        <f>"₹"&amp;TEXT(G4,"#,##0")</f>
+        <v>₹6,999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Integrate Razorpay payment: create order, checkout, verify, order success page
</commit_message>
<xml_diff>
--- a/business/pricing-calculator.xlsx
+++ b/business/pricing-calculator.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{0674D6E0-614F-4B80-828B-1369AC9A670F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F06BD3C-0D48-4615-8558-C35C34D321B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
   <sheets>
     <sheet name="pricing-calculator" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -939,7 +952,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692CD7B8-8219-4BAB-B946-0AD4DC2CA2E3}">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -956,7 +969,7 @@
     <col min="13" max="13" width="7.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -994,7 +1007,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1002,14 +1015,14 @@
         <v>450</v>
       </c>
       <c r="C2">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D2">
         <v>150</v>
       </c>
       <c r="E2">
         <f>B2+C2+D2</f>
-        <v>625</v>
+        <v>650</v>
       </c>
       <c r="F2">
         <v>3</v>
@@ -1028,18 +1041,25 @@
       </c>
       <c r="J2">
         <f>I2-E2</f>
-        <v>1334.02</v>
+        <v>1309.02</v>
       </c>
       <c r="K2" s="1">
         <f>J2/G2</f>
-        <v>0.66734367183591792</v>
+        <v>0.65483741870935464</v>
       </c>
       <c r="L2" t="str">
         <f>"₹"&amp;TEXT(G2,"#,##0")</f>
         <v>₹1,999</v>
       </c>
+      <c r="N2">
+        <v>1999</v>
+      </c>
+      <c r="O2">
+        <f>G2-N2</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1047,14 +1067,14 @@
         <v>1240</v>
       </c>
       <c r="C3">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D3">
         <v>150</v>
       </c>
       <c r="E3">
         <f>B3+C3+D3</f>
-        <v>1415</v>
+        <v>1440</v>
       </c>
       <c r="F3">
         <v>3</v>
@@ -1073,18 +1093,25 @@
       </c>
       <c r="J3">
         <f>I3-E3</f>
-        <v>2994.0200000000004</v>
+        <v>2969.0200000000004</v>
       </c>
       <c r="K3" s="1">
         <f>J3/G3</f>
-        <v>0.66548566348077365</v>
+        <v>0.65992887308290737</v>
       </c>
       <c r="L3" t="str">
         <f>"₹"&amp;TEXT(G3,"#,##0")</f>
         <v>₹4,499</v>
       </c>
+      <c r="N3">
+        <v>4499</v>
+      </c>
+      <c r="O3">
+        <f t="shared" ref="O3:O6" si="0">G3-N3</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1092,14 +1119,14 @@
         <v>1495</v>
       </c>
       <c r="C4">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D4">
         <v>150</v>
       </c>
       <c r="E4">
         <f>B4+C4+D4</f>
-        <v>1670</v>
+        <v>1695</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -1118,18 +1145,25 @@
       </c>
       <c r="J4">
         <f>I4-E4</f>
-        <v>3719.0200000000004</v>
+        <v>3694.0200000000004</v>
       </c>
       <c r="K4" s="1">
         <f>J4/G4</f>
-        <v>0.67630841971267508</v>
+        <v>0.67176213857064926</v>
       </c>
       <c r="L4" t="str">
         <f>"₹"&amp;TEXT(G4,"#,##0")</f>
         <v>₹5,499</v>
       </c>
+      <c r="N4">
+        <v>5499</v>
+      </c>
+      <c r="O4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1137,14 +1171,14 @@
         <v>1134</v>
       </c>
       <c r="C5">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D5">
         <v>150</v>
       </c>
       <c r="E5">
         <f>B5+C5+D5</f>
-        <v>1309</v>
+        <v>1314</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -1163,18 +1197,25 @@
       </c>
       <c r="J5">
         <f>I5-E5</f>
-        <v>2610.02</v>
+        <v>2605.02</v>
       </c>
       <c r="K5" s="1">
         <f>J5/G5</f>
-        <v>0.65266816704176045</v>
+        <v>0.65141785446361589</v>
       </c>
       <c r="L5" t="str">
         <f>"₹"&amp;TEXT(G5,"#,##0")</f>
         <v>₹3,999</v>
       </c>
+      <c r="N5">
+        <v>3999</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1182,14 +1223,14 @@
         <v>2100</v>
       </c>
       <c r="C6">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>150</v>
       </c>
       <c r="E6">
         <f>B6+C6+D6</f>
-        <v>2275</v>
+        <v>2280</v>
       </c>
       <c r="F6">
         <v>1.75</v>
@@ -1208,15 +1249,22 @@
       </c>
       <c r="J6">
         <f>I6-E6</f>
-        <v>1644.02</v>
+        <v>1639.02</v>
       </c>
       <c r="K6" s="1">
         <f>J6/G6</f>
-        <v>0.41110777694423606</v>
+        <v>0.4098574643660915</v>
       </c>
       <c r="L6" t="str">
         <f>"₹"&amp;TEXT(G6,"#,##0")</f>
         <v>₹3,999</v>
+      </c>
+      <c r="N6">
+        <v>3999</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add checkout gate (require login), remove all placeholder products
</commit_message>
<xml_diff>
--- a/business/pricing-calculator.xlsx
+++ b/business/pricing-calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F984C922-6B7F-42D1-A934-68AD0248A023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B228A280-2A9A-46CA-8656-8AD6E6C2C687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
@@ -1249,41 +1249,41 @@
         <v>472</v>
       </c>
       <c r="C7">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D7">
         <v>150</v>
       </c>
       <c r="E7">
         <f>B7+C7+D7</f>
-        <v>652</v>
+        <v>672</v>
       </c>
       <c r="F7">
         <v>3</v>
       </c>
       <c r="G7">
         <f>ROUNDUP((E7*F7)/500,0)*500-1</f>
-        <v>1999</v>
+        <v>2499</v>
       </c>
       <c r="H7">
         <f>G7*2%</f>
-        <v>39.980000000000004</v>
+        <v>49.980000000000004</v>
       </c>
       <c r="I7">
         <f>G7-H7</f>
-        <v>1959.02</v>
+        <v>2449.02</v>
       </c>
       <c r="J7">
         <f>I7-E7</f>
-        <v>1307.02</v>
+        <v>1777.02</v>
       </c>
       <c r="K7" s="1">
         <f>J7/G7</f>
-        <v>0.65383691845922964</v>
+        <v>0.71109243697478985</v>
       </c>
       <c r="L7" t="str">
         <f>"₹"&amp;TEXT(G7,"#,##0")</f>
-        <v>₹1,999</v>
+        <v>₹2,499</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -1294,14 +1294,14 @@
         <v>71</v>
       </c>
       <c r="C8">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D8">
         <v>150</v>
       </c>
       <c r="E8">
         <f>B8+C8+D8</f>
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="F8">
         <v>3</v>
@@ -1320,11 +1320,11 @@
       </c>
       <c r="J8">
         <f>I8-E8</f>
-        <v>728.02</v>
+        <v>708.02</v>
       </c>
       <c r="K8" s="1">
         <f>J8/G8</f>
-        <v>0.72874874874874873</v>
+        <v>0.70872872872872872</v>
       </c>
       <c r="L8" t="str">
         <f>"₹"&amp;TEXT(G8,"#,##0")</f>
@@ -1339,14 +1339,14 @@
         <v>110</v>
       </c>
       <c r="C9">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D9">
         <v>150</v>
       </c>
       <c r="E9">
         <f>B9+C9+D9</f>
-        <v>290</v>
+        <v>310</v>
       </c>
       <c r="F9">
         <v>3</v>
@@ -1365,11 +1365,11 @@
       </c>
       <c r="J9">
         <f>I9-E9</f>
-        <v>689.02</v>
+        <v>669.02</v>
       </c>
       <c r="K9" s="1">
         <f>J9/G9</f>
-        <v>0.68970970970970968</v>
+        <v>0.66968968968968967</v>
       </c>
       <c r="L9" t="str">
         <f>"₹"&amp;TEXT(G9,"#,##0")</f>

</xml_diff>

<commit_message>
Add Collections hover dropdown, remove Bridal from navbar
</commit_message>
<xml_diff>
--- a/business/pricing-calculator.xlsx
+++ b/business/pricing-calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahujadiv\Desktop\Team\Automations\JBG\jewels-by-geetika\business\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B228A280-2A9A-46CA-8656-8AD6E6C2C687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45EAE58C-4359-41DE-BE8B-0A99C179132A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3EA1E2F3-88D9-406C-AEBC-3B66D1D0E7C6}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Product Name</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>Sunehri</t>
+  </si>
+  <si>
+    <t>Antara</t>
   </si>
 </sst>
 </file>
@@ -961,7 +964,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{692CD7B8-8219-4BAB-B946-0AD4DC2CA2E3}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -1376,6 +1379,51 @@
         <v>₹999</v>
       </c>
     </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10">
+        <v>1070</v>
+      </c>
+      <c r="C10">
+        <v>50</v>
+      </c>
+      <c r="D10">
+        <v>150</v>
+      </c>
+      <c r="E10">
+        <f>B10+C10+D10</f>
+        <v>1270</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <f>ROUNDUP((E10*F10)/500,0)*500-1</f>
+        <v>3999</v>
+      </c>
+      <c r="H10">
+        <f>G10*2%</f>
+        <v>79.98</v>
+      </c>
+      <c r="I10">
+        <f>G10-H10</f>
+        <v>3919.02</v>
+      </c>
+      <c r="J10">
+        <f>I10-E10</f>
+        <v>2649.02</v>
+      </c>
+      <c r="K10" s="1">
+        <f>J10/G10</f>
+        <v>0.66242060515128787</v>
+      </c>
+      <c r="L10" t="str">
+        <f>"₹"&amp;TEXT(G10,"#,##0")</f>
+        <v>₹3,999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>